<commit_message>
fix(seo): perbaiki canonical dan og:url landing page ke site.donkap.space
Semua halaman landing sebelumnya punya canonical yang mengarah ke donkap.space
(domain app/login), bukan site.donkap.space (domain landing page sebenarnya).
Ini menyebabkan Google disuruh index halaman login app sebagai konten utama.

Fixes task #4 — konsolidasi SEO authority ke domain yang benar.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/action_plan_assigned.xlsx
+++ b/action_plan_assigned.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 Master Action Plan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📅 Timeline" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="✅ Tracker Harian" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="💰 MRR Projection" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="👥 Role Assignment" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔗 Dependency Map" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="📊 Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📋 Master Action Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📅 Timeline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="✅ Tracker Harian" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="💰 MRR Projection" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="👥 Role Assignment" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="🔗 Dependency Map" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'📋 Master Action Plan'!$B$4:$L$43</definedName>
@@ -1929,12 +1929,12 @@
       </c>
       <c r="K9" s="45" t="inlineStr">
         <is>
-          <t>⬜ Belum Mulai</t>
+          <t>✅ Selesai</t>
         </is>
       </c>
       <c r="L9" s="45" t="inlineStr">
         <is>
-          <t>Redirect site.donkap.space → donkap.space. SEO authority sekarang terbelah</t>
+          <t>Canonical + og:url semua halaman landing diperbaiki ke site.donkap.space. Sitemap sudah benar.</t>
         </is>
       </c>
       <c r="M9" s="114" t="inlineStr">

</xml_diff>

<commit_message>
chore: mark task #9 selesai — post FB Group UMKM
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/action_plan_assigned.xlsx
+++ b/action_plan_assigned.xlsx
@@ -2349,12 +2349,12 @@
       </c>
       <c r="K14" s="51" t="inlineStr">
         <is>
-          <t>⬜ Belum Mulai</t>
+          <t>✅ Selesai</t>
         </is>
       </c>
       <c r="L14" s="51" t="inlineStr">
         <is>
-          <t>BUKAN promosi. Post tips cara rekap absensi. Mention Donkap di akhir</t>
+          <t>Post value content tips absensi sudah dilakukan di 3 FB Group UMKM besar oleh founder.</t>
         </is>
       </c>
       <c r="M14" s="114" t="inlineStr">

</xml_diff>

<commit_message>
feat(pricing): naikkan harga Pro dari Rp29rb ke Rp79rb
Hapus testimonial yang menyebut harga lama agar tidak menyesatkan.
Update WA link CTA sesuai harga baru.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/action_plan_assigned.xlsx
+++ b/action_plan_assigned.xlsx
@@ -2618,12 +2618,12 @@
       </c>
       <c r="K18" s="45" t="inlineStr">
         <is>
-          <t>⬜ Belum Mulai</t>
+          <t>✅ Selesai</t>
         </is>
       </c>
       <c r="L18" s="45" t="inlineStr">
         <is>
-          <t>Rp29rb terlalu murah. 2.7x MRR lebih baik. Masih sangat terjangkau untuk bisnis</t>
+          <t>Harga Pro diubah ke Rp79rb di landing page. Testimonial yang menyebut 29rb dihapus.</t>
         </is>
       </c>
       <c r="M18" s="114" t="inlineStr">

</xml_diff>

<commit_message>
chore: mark task #19 selesai — daftar Capterra
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/action_plan_assigned.xlsx
+++ b/action_plan_assigned.xlsx
@@ -3206,12 +3206,12 @@
       </c>
       <c r="K25" s="51" t="inlineStr">
         <is>
-          <t>⬜ Belum Mulai</t>
+          <t>✅ Selesai</t>
         </is>
       </c>
       <c r="L25" s="51" t="inlineStr">
         <is>
-          <t>Backlink gratis. Capterra dan G2 punya listing gratis untuk startup</t>
+          <t>Sudah daftar di Capterra. G2 dan direktori UMKM lainnya bisa menyusul.</t>
         </is>
       </c>
       <c r="M25" s="114" t="inlineStr">

</xml_diff>

<commit_message>
feat(landing): tambah tier harga Bisnis & Pro (task #18)
- Pricing section diubah dari 2 tier menjadi 3 tier:
  - Gratis: Rp 0, hingga 10 karyawan
  - Bisnis: Rp 79rb/bulan, hingga 50 karyawan (rename dari "Pro")
  - Pro: Rp 199rb/bulan, karyawan unlimited + multi-lokasi + fitur premium
- Tambah task #36-39 di roadmap: ide fitur Pro (notif telat, dashboard cabang, estimasi lembur, approval workflow)
- Task #18 ditandai selesai di action plan

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/action_plan_assigned.xlsx
+++ b/action_plan_assigned.xlsx
@@ -1484,7 +1484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="B1:S49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="95" min="1" max="1"/>
@@ -3122,12 +3122,12 @@
       </c>
       <c r="K24" s="51" t="inlineStr">
         <is>
-          <t>⬜ Belum Mulai</t>
+          <t>✅ Selesai</t>
         </is>
       </c>
       <c r="L24" s="51" t="inlineStr">
         <is>
-          <t>Tier terlalu sedikit. Feature gating yang jelas per tier</t>
+          <t>Landing page diupdate: 3 tier (Gratis/Bisnis Rp79rb/Pro Rp199rb). Feature gating backend belum diimplementasi.</t>
         </is>
       </c>
       <c r="M24" s="114" t="inlineStr">
@@ -4625,6 +4625,209 @@
       <c r="S43" s="114" t="inlineStr">
         <is>
           <t>Internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  💡 FITUR PRO (ROADMAP IDEAS — dari brainstorm Jun 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="0" t="n">
+        <v>36</v>
+      </c>
+      <c r="C46" s="0" t="inlineStr">
+        <is>
+          <t>Notifikasi telat real-time ke owner</t>
+        </is>
+      </c>
+      <c r="D46" s="0" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E46" s="0" t="inlineStr">
+        <is>
+          <t>🟠 TINGGI</t>
+        </is>
+      </c>
+      <c r="F46" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H46" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="I46" s="0" t="inlineStr">
+        <is>
+          <t>1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="J46" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="K46" s="0" t="inlineStr">
+        <is>
+          <t>⬜ Belum Mulai</t>
+        </is>
+      </c>
+      <c r="L46" s="0" t="inlineStr">
+        <is>
+          <t>Alert email/WA ke owner kalau karyawan belum check-in 15 menit setelah jam mulai kerja. Owner UMKM paling sensitif sama masalah ini.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="0" t="n">
+        <v>37</v>
+      </c>
+      <c r="C47" s="0" t="inlineStr">
+        <is>
+          <t>Dashboard per-cabang (multi-lokasi)</t>
+        </is>
+      </c>
+      <c r="D47" s="0" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E47" s="0" t="inlineStr">
+        <is>
+          <t>🟠 TINGGI</t>
+        </is>
+      </c>
+      <c r="F47" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="G47" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H47" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="I47" s="0" t="inlineStr">
+        <is>
+          <t>1 Sep 2026</t>
+        </is>
+      </c>
+      <c r="J47" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="K47" s="0" t="inlineStr">
+        <is>
+          <t>⬜ Belum Mulai</t>
+        </is>
+      </c>
+      <c r="L47" s="0" t="inlineStr">
+        <is>
+          <t>Owner dengan banyak outlet bisa lihat kehadiran per-cabang sekaligus. Backend multi_location sudah ada, tinggal UI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="0" t="n">
+        <v>38</v>
+      </c>
+      <c r="C48" s="0" t="inlineStr">
+        <is>
+          <t>Laporan estimasi biaya lembur otomatis</t>
+        </is>
+      </c>
+      <c r="D48" s="0" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E48" s="0" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="F48" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H48" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="I48" s="0" t="inlineStr">
+        <is>
+          <t>1 Okt 2026</t>
+        </is>
+      </c>
+      <c r="J48" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="K48" s="0" t="inlineStr">
+        <is>
+          <t>⬜ Belum Mulai</t>
+        </is>
+      </c>
+      <c r="L48" s="0" t="inlineStr">
+        <is>
+          <t>Hitung otomatis estimasi biaya lembur per karyawan berdasarkan rate yang diset admin. UMKM sering pusing rekap lembur manual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="0" t="n">
+        <v>39</v>
+      </c>
+      <c r="C49" s="0" t="inlineStr">
+        <is>
+          <t>Approval workflow bertingkat untuk izin/cuti</t>
+        </is>
+      </c>
+      <c r="D49" s="0" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E49" s="0" t="inlineStr">
+        <is>
+          <t>🟡 MEDIUM</t>
+        </is>
+      </c>
+      <c r="F49" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G49" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H49" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="I49" s="0" t="inlineStr">
+        <is>
+          <t>1 Okt 2026</t>
+        </is>
+      </c>
+      <c r="J49" s="0" t="inlineStr">
+        <is>
+          <t>Dev</t>
+        </is>
+      </c>
+      <c r="K49" s="0" t="inlineStr">
+        <is>
+          <t>⬜ Belum Mulai</t>
+        </is>
+      </c>
+      <c r="L49" s="0" t="inlineStr">
+        <is>
+          <t>Karyawan request → manager approve → owner final approve. Saat ini approval flat. Penting untuk bisnis dengan struktur tim.</t>
         </is>
       </c>
     </row>

</xml_diff>